<commit_message>
Restructure site: minimal homepage + dropdown nav + new pages (bikes/specs/sizes/faq/guides/gallery/community/reviews/contact)
</commit_message>
<xml_diff>
--- a/spinz-shipping-comparison.xlsx
+++ b/spinz-shipping-comparison.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="השוואת חברות" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="סימולטור עלות חודשית" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="שאלות לחברות" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="השוואת חברות" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="סימולטור עלות חודשית" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="שאלות לחברות" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -195,7 +195,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" readingOrder="2"/>
@@ -311,6 +311,16 @@
     <xf numFmtId="0" fontId="10" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" readingOrder="2"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -676,7 +686,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X19"/>
+  <dimension ref="A1:AI25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -746,6 +756,61 @@
           <t>── פיננסי ──</t>
         </is>
       </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>── עלויות קבועות ──</t>
+        </is>
+      </c>
+      <c r="Z4" t="inlineStr">
+        <is>
+          <t>נשלח בקשת מחיר</t>
+        </is>
+      </c>
+      <c r="AA4" t="inlineStr">
+        <is>
+          <t>נשלח בקשת מחיר</t>
+        </is>
+      </c>
+      <c r="AB4" t="inlineStr">
+        <is>
+          <t>נשלח בקשת מחיר</t>
+        </is>
+      </c>
+      <c r="AC4" t="inlineStr">
+        <is>
+          <t>נשלח בקשת מחיר</t>
+        </is>
+      </c>
+      <c r="AD4" t="inlineStr">
+        <is>
+          <t>נשלח בקשת מחיר</t>
+        </is>
+      </c>
+      <c r="AE4" t="inlineStr">
+        <is>
+          <t>נשלח בקשת מחיר</t>
+        </is>
+      </c>
+      <c r="AF4" t="inlineStr">
+        <is>
+          <t>נשלח בקשת מחיר</t>
+        </is>
+      </c>
+      <c r="AG4" t="inlineStr">
+        <is>
+          <t>נשלח בקשת מחיר</t>
+        </is>
+      </c>
+      <c r="AH4" t="inlineStr">
+        <is>
+          <t>נשלח בקשת מחיר</t>
+        </is>
+      </c>
+      <c r="AI4" t="inlineStr">
+        <is>
+          <t>נשלח בקשת מחיר</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="40" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
@@ -866,6 +931,21 @@
       <c r="X5" s="4" t="inlineStr">
         <is>
           <t>תנאי תשלום (שוטף +?)</t>
+        </is>
+      </c>
+      <c r="Y5" t="inlineStr">
+        <is>
+          <t>דמי מנוי חודשי (₪)</t>
+        </is>
+      </c>
+      <c r="Z5" t="inlineStr">
+        <is>
+          <t>מינימום חיוב חודשי (₪)</t>
+        </is>
+      </c>
+      <c r="AA5" t="inlineStr">
+        <is>
+          <t>עלויות קבועות סה"כ (₪)</t>
         </is>
       </c>
     </row>
@@ -898,6 +978,11 @@
       <c r="V6" s="9" t="inlineStr"/>
       <c r="W6" s="10" t="inlineStr"/>
       <c r="X6" s="10" t="inlineStr"/>
+      <c r="AD6" t="inlineStr">
+        <is>
+          <t>✅ 25/05/2026</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="20" customHeight="1">
       <c r="A7" s="11" t="inlineStr">
@@ -905,7 +990,11 @@
           <t>HFD שליחויות ולוגיסטיקה</t>
         </is>
       </c>
-      <c r="B7" s="12" t="inlineStr"/>
+      <c r="B7" s="12" t="inlineStr">
+        <is>
+          <t>❌ לא רלוונטי — לא מפיצים חבילות במידות/משקל של האופניים</t>
+        </is>
+      </c>
       <c r="C7" s="12" t="inlineStr"/>
       <c r="D7" s="12" t="inlineStr"/>
       <c r="E7" s="12" t="inlineStr"/>
@@ -928,6 +1017,21 @@
       <c r="V7" s="15" t="inlineStr"/>
       <c r="W7" s="16" t="inlineStr"/>
       <c r="X7" s="16" t="inlineStr"/>
+      <c r="AD7" t="inlineStr">
+        <is>
+          <t>✅ 25/05/2026</t>
+        </is>
+      </c>
+      <c r="AF7" t="inlineStr">
+        <is>
+          <t>✅ 26/05/2026</t>
+        </is>
+      </c>
+      <c r="AI7" t="inlineStr">
+        <is>
+          <t>✅ 31/05/2026</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="20" customHeight="1">
       <c r="A8" s="5" t="inlineStr">
@@ -958,6 +1062,16 @@
       <c r="V8" s="9" t="inlineStr"/>
       <c r="W8" s="10" t="inlineStr"/>
       <c r="X8" s="10" t="inlineStr"/>
+      <c r="AD8" t="inlineStr">
+        <is>
+          <t>✅ 25/05/2026</t>
+        </is>
+      </c>
+      <c r="AE8" t="inlineStr">
+        <is>
+          <t>✅ 25/05/2026</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="20" customHeight="1">
       <c r="A9" s="11" t="inlineStr">
@@ -965,19 +1079,41 @@
           <t>צ'יטה שליחויות (Cheetah)</t>
         </is>
       </c>
-      <c r="B9" s="12" t="inlineStr"/>
-      <c r="C9" s="12" t="inlineStr"/>
-      <c r="D9" s="12" t="inlineStr"/>
+      <c r="B9" s="12" t="n">
+        <v>70</v>
+      </c>
+      <c r="C9" s="12" t="inlineStr">
+        <is>
+          <t>כלול</t>
+        </is>
+      </c>
+      <c r="D9" s="12" t="inlineStr">
+        <is>
+          <t>+50%</t>
+        </is>
+      </c>
       <c r="E9" s="12" t="inlineStr"/>
       <c r="F9" s="12" t="inlineStr"/>
-      <c r="G9" s="12" t="inlineStr"/>
+      <c r="G9" s="12" t="inlineStr">
+        <is>
+          <t>+100%</t>
+        </is>
+      </c>
       <c r="H9" s="13" t="inlineStr"/>
       <c r="I9" s="13" t="inlineStr"/>
       <c r="J9" s="13" t="inlineStr"/>
       <c r="K9" s="13" t="inlineStr"/>
       <c r="L9" s="13" t="inlineStr"/>
-      <c r="M9" s="14" t="inlineStr"/>
-      <c r="N9" s="14" t="inlineStr"/>
+      <c r="M9" s="14" t="inlineStr">
+        <is>
+          <t>140 ₪/חודש (כל המשלוחים)</t>
+        </is>
+      </c>
+      <c r="N9" s="14" t="inlineStr">
+        <is>
+          <t>לפי תנאי ההסכם</t>
+        </is>
+      </c>
       <c r="O9" s="14" t="inlineStr"/>
       <c r="P9" s="14" t="inlineStr"/>
       <c r="Q9" s="15" t="inlineStr"/>
@@ -988,6 +1124,25 @@
       <c r="V9" s="15" t="inlineStr"/>
       <c r="W9" s="16" t="inlineStr"/>
       <c r="X9" s="16" t="inlineStr"/>
+      <c r="Y9" t="n">
+        <v>120</v>
+      </c>
+      <c r="Z9" t="n">
+        <v>700</v>
+      </c>
+      <c r="AA9" t="n">
+        <v>960</v>
+      </c>
+      <c r="AD9" t="inlineStr">
+        <is>
+          <t>✅ 25/05/2026</t>
+        </is>
+      </c>
+      <c r="AI9" t="inlineStr">
+        <is>
+          <t>✅ 31/05/2026</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="5" t="inlineStr">
@@ -1018,6 +1173,21 @@
       <c r="V10" s="9" t="inlineStr"/>
       <c r="W10" s="10" t="inlineStr"/>
       <c r="X10" s="10" t="inlineStr"/>
+      <c r="AD10" t="inlineStr">
+        <is>
+          <t>✅ 25/05/2026</t>
+        </is>
+      </c>
+      <c r="AF10" t="inlineStr">
+        <is>
+          <t>✅ 26/05/2026</t>
+        </is>
+      </c>
+      <c r="AI10" t="inlineStr">
+        <is>
+          <t>✅ 31/05/2026</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="11" t="inlineStr">
@@ -1048,6 +1218,11 @@
       <c r="V11" s="15" t="inlineStr"/>
       <c r="W11" s="16" t="inlineStr"/>
       <c r="X11" s="16" t="inlineStr"/>
+      <c r="AD11" t="inlineStr">
+        <is>
+          <t>✅ 25/05/2026</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="5" t="inlineStr">
@@ -1078,6 +1253,11 @@
       <c r="V12" s="9" t="inlineStr"/>
       <c r="W12" s="10" t="inlineStr"/>
       <c r="X12" s="10" t="inlineStr"/>
+      <c r="AD12" t="inlineStr">
+        <is>
+          <t>✅ 25/05/2026</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="20" customHeight="1">
       <c r="A13" s="11" t="inlineStr">
@@ -1085,7 +1265,11 @@
           <t>הום דילברי (Home Delivery)</t>
         </is>
       </c>
-      <c r="B13" s="12" t="inlineStr"/>
+      <c r="B13" s="12" t="inlineStr">
+        <is>
+          <t>⚠️ לא אומתה כחברה פעילה — לא נמצא אתר/מייל</t>
+        </is>
+      </c>
       <c r="C13" s="12" t="inlineStr"/>
       <c r="D13" s="12" t="inlineStr"/>
       <c r="E13" s="12" t="inlineStr"/>
@@ -1108,6 +1292,16 @@
       <c r="V13" s="15" t="inlineStr"/>
       <c r="W13" s="16" t="inlineStr"/>
       <c r="X13" s="16" t="inlineStr"/>
+      <c r="AG13" t="inlineStr">
+        <is>
+          <t>✅ 31/05/2026</t>
+        </is>
+      </c>
+      <c r="AH13" t="inlineStr">
+        <is>
+          <t>✅ 31/05/2026</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="20" customHeight="1">
       <c r="A14" s="5" t="inlineStr">
@@ -1115,7 +1309,11 @@
           <t>יונט קארגו</t>
         </is>
       </c>
-      <c r="B14" s="6" t="inlineStr"/>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>⚠️ לא אומתה כחברה פעילה — לא נמצא אתר/מייל</t>
+        </is>
+      </c>
       <c r="C14" s="6" t="inlineStr"/>
       <c r="D14" s="6" t="inlineStr"/>
       <c r="E14" s="6" t="inlineStr"/>
@@ -1138,6 +1336,16 @@
       <c r="V14" s="9" t="inlineStr"/>
       <c r="W14" s="10" t="inlineStr"/>
       <c r="X14" s="10" t="inlineStr"/>
+      <c r="AD14" t="inlineStr">
+        <is>
+          <t>✅ 25/05/2026</t>
+        </is>
+      </c>
+      <c r="AE14" t="inlineStr">
+        <is>
+          <t>✅ 25/05/2026</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="20" customHeight="1">
       <c r="A15" s="11" t="inlineStr">
@@ -1145,7 +1353,11 @@
           <t>נאוי לוגיסטיקה</t>
         </is>
       </c>
-      <c r="B15" s="12" t="inlineStr"/>
+      <c r="B15" s="12" t="inlineStr">
+        <is>
+          <t>⚠️ לא אומתה כחברה פעילה — לא נמצא אתר/מייל</t>
+        </is>
+      </c>
       <c r="C15" s="12" t="inlineStr"/>
       <c r="D15" s="12" t="inlineStr"/>
       <c r="E15" s="12" t="inlineStr"/>
@@ -1168,6 +1380,11 @@
       <c r="V15" s="15" t="inlineStr"/>
       <c r="W15" s="16" t="inlineStr"/>
       <c r="X15" s="16" t="inlineStr"/>
+      <c r="AI15" t="inlineStr">
+        <is>
+          <t>✅ 31/05/2026</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="20" customHeight="1">
       <c r="A16" s="5" t="inlineStr">
@@ -1175,7 +1392,11 @@
           <t>ATA לוגיסטיקה</t>
         </is>
       </c>
-      <c r="B16" s="6" t="inlineStr"/>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>⚠️ לא אומתה כחברה פעילה — לא נמצא אתר/מייל</t>
+        </is>
+      </c>
       <c r="C16" s="6" t="inlineStr"/>
       <c r="D16" s="6" t="inlineStr"/>
       <c r="E16" s="6" t="inlineStr"/>
@@ -1198,6 +1419,11 @@
       <c r="V16" s="9" t="inlineStr"/>
       <c r="W16" s="10" t="inlineStr"/>
       <c r="X16" s="10" t="inlineStr"/>
+      <c r="AI16" t="inlineStr">
+        <is>
+          <t>✅ 31/05/2026</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="20" customHeight="1">
       <c r="A17" s="11" t="inlineStr">
@@ -1228,6 +1454,11 @@
       <c r="V17" s="15" t="inlineStr"/>
       <c r="W17" s="16" t="inlineStr"/>
       <c r="X17" s="16" t="inlineStr"/>
+      <c r="AD17" t="inlineStr">
+        <is>
+          <t>✅ 25/05/2026</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="20" customHeight="1">
       <c r="A18" s="5" t="inlineStr">
@@ -1235,7 +1466,11 @@
           <t>Speedex</t>
         </is>
       </c>
-      <c r="B18" s="6" t="inlineStr"/>
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>⚠️ לא אומתה כחברה פעילה — לא נמצא אתר/מייל</t>
+        </is>
+      </c>
       <c r="C18" s="6" t="inlineStr"/>
       <c r="D18" s="6" t="inlineStr"/>
       <c r="E18" s="6" t="inlineStr"/>
@@ -1288,6 +1523,290 @@
       <c r="V19" s="15" t="inlineStr"/>
       <c r="W19" s="16" t="inlineStr"/>
       <c r="X19" s="16" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="41" t="inlineStr">
+        <is>
+          <t>Tigger Delivery</t>
+        </is>
+      </c>
+      <c r="B20" s="41" t="n">
+        <v>80</v>
+      </c>
+      <c r="C20" s="41" t="inlineStr">
+        <is>
+          <t>כלול במחיר</t>
+        </is>
+      </c>
+      <c r="D20" s="41" t="inlineStr">
+        <is>
+          <t>100 ש"ח — אילת, ערבה, ים המלח, דימונה</t>
+        </is>
+      </c>
+      <c r="E20" s="41" t="n"/>
+      <c r="F20" s="41" t="n"/>
+      <c r="G20" s="41" t="n"/>
+      <c r="H20" s="42" t="inlineStr">
+        <is>
+          <t>עד 5</t>
+        </is>
+      </c>
+      <c r="I20" s="42" t="inlineStr">
+        <is>
+          <t>עד 5</t>
+        </is>
+      </c>
+      <c r="J20" s="42" t="n"/>
+      <c r="K20" s="42" t="n"/>
+      <c r="L20" s="42" t="inlineStr">
+        <is>
+          <t>בנק 50 משלוחים (ללא הגבלת זמן)</t>
+        </is>
+      </c>
+      <c r="M20" s="43" t="n"/>
+      <c r="N20" s="43" t="n"/>
+      <c r="O20" s="43" t="n"/>
+      <c r="P20" s="43" t="n"/>
+      <c r="Q20" s="44" t="n"/>
+      <c r="R20" s="44" t="n"/>
+      <c r="S20" s="44" t="n"/>
+      <c r="T20" s="44" t="n"/>
+      <c r="U20" s="44" t="n"/>
+      <c r="V20" s="44" t="n"/>
+      <c r="W20" s="44" t="n"/>
+      <c r="X20" s="44" t="inlineStr">
+        <is>
+          <t>לא כולל מע"מ</t>
+        </is>
+      </c>
+      <c r="Y20" s="44" t="n"/>
+      <c r="Z20" s="44" t="inlineStr">
+        <is>
+          <t>אין מינימום חודשי — בנק 50 משלוחים</t>
+        </is>
+      </c>
+      <c r="AA20" s="44" t="n"/>
+      <c r="AB20" s="44" t="n"/>
+      <c r="AC20" s="44" t="n"/>
+      <c r="AD20" s="44" t="n"/>
+      <c r="AE20" s="44" t="n"/>
+      <c r="AF20" s="44" t="n"/>
+      <c r="AG20" s="44" t="inlineStr">
+        <is>
+          <t>✅ 31/05/2026</t>
+        </is>
+      </c>
+      <c r="AH20" s="44" t="inlineStr">
+        <is>
+          <t>✅ 31/05/2026</t>
+        </is>
+      </c>
+      <c r="AI20" s="44" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="45" t="inlineStr">
+        <is>
+          <t>יהב לוגיסטיקה</t>
+        </is>
+      </c>
+      <c r="B21" s="45" t="n"/>
+      <c r="C21" s="45" t="n"/>
+      <c r="D21" s="45" t="n"/>
+      <c r="E21" s="45" t="n"/>
+      <c r="F21" s="45" t="n"/>
+      <c r="G21" s="45" t="n"/>
+      <c r="H21" s="46" t="n"/>
+      <c r="I21" s="46" t="n"/>
+      <c r="J21" s="46" t="n"/>
+      <c r="K21" s="46" t="n"/>
+      <c r="L21" s="46" t="n"/>
+      <c r="M21" s="47" t="n"/>
+      <c r="N21" s="47" t="n"/>
+      <c r="O21" s="47" t="n"/>
+      <c r="P21" s="47" t="n"/>
+      <c r="Q21" s="48" t="n"/>
+      <c r="R21" s="48" t="n"/>
+      <c r="S21" s="48" t="n"/>
+      <c r="T21" s="48" t="n"/>
+      <c r="U21" s="48" t="n"/>
+      <c r="V21" s="48" t="n"/>
+      <c r="W21" s="48" t="n"/>
+      <c r="X21" s="48" t="n"/>
+      <c r="Y21" s="48" t="n"/>
+      <c r="Z21" s="48" t="n"/>
+      <c r="AA21" s="48" t="n"/>
+      <c r="AB21" s="48" t="n"/>
+      <c r="AC21" s="48" t="n"/>
+      <c r="AD21" s="48" t="n"/>
+      <c r="AE21" s="48" t="n"/>
+      <c r="AF21" s="48" t="n"/>
+      <c r="AG21" s="48" t="n"/>
+      <c r="AH21" s="48" t="n"/>
+      <c r="AI21" s="48" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="41" t="inlineStr">
+        <is>
+          <t>אמגון</t>
+        </is>
+      </c>
+      <c r="B22" s="41" t="n"/>
+      <c r="C22" s="41" t="n"/>
+      <c r="D22" s="41" t="n"/>
+      <c r="E22" s="41" t="n"/>
+      <c r="F22" s="41" t="n"/>
+      <c r="G22" s="41" t="n"/>
+      <c r="H22" s="42" t="n"/>
+      <c r="I22" s="42" t="n"/>
+      <c r="J22" s="42" t="n"/>
+      <c r="K22" s="42" t="n"/>
+      <c r="L22" s="42" t="n"/>
+      <c r="M22" s="43" t="n"/>
+      <c r="N22" s="43" t="n"/>
+      <c r="O22" s="43" t="n"/>
+      <c r="P22" s="43" t="n"/>
+      <c r="Q22" s="44" t="n"/>
+      <c r="R22" s="44" t="n"/>
+      <c r="S22" s="44" t="n"/>
+      <c r="T22" s="44" t="n"/>
+      <c r="U22" s="44" t="n"/>
+      <c r="V22" s="44" t="n"/>
+      <c r="W22" s="44" t="n"/>
+      <c r="X22" s="44" t="n"/>
+      <c r="Y22" s="44" t="n"/>
+      <c r="Z22" s="44" t="n"/>
+      <c r="AA22" s="44" t="n"/>
+      <c r="AB22" s="44" t="n"/>
+      <c r="AC22" s="44" t="n"/>
+      <c r="AD22" s="44" t="n"/>
+      <c r="AE22" s="44" t="n"/>
+      <c r="AF22" s="44" t="n"/>
+      <c r="AG22" s="44" t="n"/>
+      <c r="AH22" s="44" t="n"/>
+      <c r="AI22" s="44" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="45" t="inlineStr">
+        <is>
+          <t>רצ פלוס שליחויות</t>
+        </is>
+      </c>
+      <c r="B23" s="45" t="n"/>
+      <c r="C23" s="45" t="n"/>
+      <c r="D23" s="45" t="n"/>
+      <c r="E23" s="45" t="n"/>
+      <c r="F23" s="45" t="n"/>
+      <c r="G23" s="45" t="n"/>
+      <c r="H23" s="46" t="n"/>
+      <c r="I23" s="46" t="n"/>
+      <c r="J23" s="46" t="n"/>
+      <c r="K23" s="46" t="n"/>
+      <c r="L23" s="46" t="n"/>
+      <c r="M23" s="47" t="n"/>
+      <c r="N23" s="47" t="n"/>
+      <c r="O23" s="47" t="n"/>
+      <c r="P23" s="47" t="n"/>
+      <c r="Q23" s="48" t="n"/>
+      <c r="R23" s="48" t="n"/>
+      <c r="S23" s="48" t="n"/>
+      <c r="T23" s="48" t="n"/>
+      <c r="U23" s="48" t="n"/>
+      <c r="V23" s="48" t="n"/>
+      <c r="W23" s="48" t="n"/>
+      <c r="X23" s="48" t="n"/>
+      <c r="Y23" s="48" t="n"/>
+      <c r="Z23" s="48" t="n"/>
+      <c r="AA23" s="48" t="n"/>
+      <c r="AB23" s="48" t="n"/>
+      <c r="AC23" s="48" t="n"/>
+      <c r="AD23" s="48" t="n"/>
+      <c r="AE23" s="48" t="n"/>
+      <c r="AF23" s="48" t="n"/>
+      <c r="AG23" s="48" t="n"/>
+      <c r="AH23" s="48" t="n"/>
+      <c r="AI23" s="48" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="41" t="inlineStr">
+        <is>
+          <t>GCX</t>
+        </is>
+      </c>
+      <c r="B24" s="41" t="n"/>
+      <c r="C24" s="41" t="n"/>
+      <c r="D24" s="41" t="n"/>
+      <c r="E24" s="41" t="n"/>
+      <c r="F24" s="41" t="n"/>
+      <c r="G24" s="41" t="n"/>
+      <c r="H24" s="42" t="n"/>
+      <c r="I24" s="42" t="n"/>
+      <c r="J24" s="42" t="n"/>
+      <c r="K24" s="42" t="n"/>
+      <c r="L24" s="42" t="n"/>
+      <c r="M24" s="43" t="n"/>
+      <c r="N24" s="43" t="n"/>
+      <c r="O24" s="43" t="n"/>
+      <c r="P24" s="43" t="n"/>
+      <c r="Q24" s="44" t="n"/>
+      <c r="R24" s="44" t="n"/>
+      <c r="S24" s="44" t="n"/>
+      <c r="T24" s="44" t="n"/>
+      <c r="U24" s="44" t="n"/>
+      <c r="V24" s="44" t="n"/>
+      <c r="W24" s="44" t="n"/>
+      <c r="X24" s="44" t="n"/>
+      <c r="Y24" s="44" t="n"/>
+      <c r="Z24" s="44" t="n"/>
+      <c r="AA24" s="44" t="n"/>
+      <c r="AB24" s="44" t="n"/>
+      <c r="AC24" s="44" t="n"/>
+      <c r="AD24" s="44" t="n"/>
+      <c r="AE24" s="44" t="n"/>
+      <c r="AF24" s="44" t="n"/>
+      <c r="AG24" s="44" t="n"/>
+      <c r="AH24" s="44" t="n"/>
+      <c r="AI24" s="44" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="45" t="inlineStr">
+        <is>
+          <t>Gaash Worldwide</t>
+        </is>
+      </c>
+      <c r="B25" s="45" t="n"/>
+      <c r="C25" s="45" t="n"/>
+      <c r="D25" s="45" t="n"/>
+      <c r="E25" s="45" t="n"/>
+      <c r="F25" s="45" t="n"/>
+      <c r="G25" s="45" t="n"/>
+      <c r="H25" s="46" t="n"/>
+      <c r="I25" s="46" t="n"/>
+      <c r="J25" s="46" t="n"/>
+      <c r="K25" s="46" t="n"/>
+      <c r="L25" s="46" t="n"/>
+      <c r="M25" s="47" t="n"/>
+      <c r="N25" s="47" t="n"/>
+      <c r="O25" s="47" t="n"/>
+      <c r="P25" s="47" t="n"/>
+      <c r="Q25" s="48" t="n"/>
+      <c r="R25" s="48" t="n"/>
+      <c r="S25" s="48" t="n"/>
+      <c r="T25" s="48" t="n"/>
+      <c r="U25" s="48" t="n"/>
+      <c r="V25" s="48" t="n"/>
+      <c r="W25" s="48" t="n"/>
+      <c r="X25" s="48" t="n"/>
+      <c r="Y25" s="48" t="n"/>
+      <c r="Z25" s="48" t="n"/>
+      <c r="AA25" s="48" t="n"/>
+      <c r="AB25" s="48" t="n"/>
+      <c r="AC25" s="48" t="n"/>
+      <c r="AD25" s="48" t="n"/>
+      <c r="AE25" s="48" t="n"/>
+      <c r="AF25" s="48" t="n"/>
+      <c r="AG25" s="48" t="n"/>
+      <c r="AH25" s="48" t="n"/>
+      <c r="AI25" s="48" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="7">

</xml_diff>